<commit_message>
Address review: value metric risk, GM caveat, A/B positioning
</commit_message>
<xml_diff>
--- a/day22_monetization_model.xlsx
+++ b/day22_monetization_model.xlsx
@@ -3991,6 +3991,11 @@
         <f>IF(B19=0,0,(B19-B5)/B19)</f>
         <v/>
       </c>
+      <c r="D21" s="48" t="inlineStr">
+        <is>
+          <t>GM 76,7% là GM TRỰC TIẾP (chưa gồm Overhead, 1_Cost_Job S8 = 0), nên cao hơn benchmark 53–65% (ICONIQ/Bessemer). Điền S8 để xem GM sau overhead ở 1_Cost_Job B67.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="45">
       <c r="A22" s="14" t="inlineStr">
@@ -5645,7 +5650,7 @@
       </c>
       <c r="B31" s="46" t="inlineStr">
         <is>
-          <t>Không lệch: model gợi ý OUTCOME (Attribution 7/10, Autonomy 7/10 — cả hai sát ngưỡng 7)</t>
+          <t>Không lệch gợi ý (OUTCOME; Attribution 7/10, Autonomy 7/10, cả hai sát ngưỡng). Rủi ro thị trường: SME Việt Nam quen trả theo gói cố định hoặc theo mức dùng hơn là theo kết quả. Dự phòng: nếu pilot cho thấy shop ngại, chuyển sang Hybrid (phí nền nhỏ + $/job).</t>
         </is>
       </c>
     </row>

</xml_diff>